<commit_message>
Add Yahoo trade lookup and cumulative opportunity allocations
</commit_message>
<xml_diff>
--- a/templates/onepiece-trade-import-template.xlsx
+++ b/templates/onepiece-trade-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trades" sheetId="1" r:id="R280bad0b5f24443a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R292cea8be1524779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trades" sheetId="1" r:id="Rd67291f8e4f2493b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R451be3dcfe764eb9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -305,6 +305,7 @@
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="27" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -332,6 +333,9 @@
       </x:c>
       <x:c r="E2" s="1"/>
       <x:c r="F2" s="1"/>
+      <x:c r="G2" s="4" t="str">
+        <x:v>Yahoo Finance Code</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="6" t="str">
@@ -348,6 +352,9 @@
       </x:c>
       <x:c r="E3" s="1"/>
       <x:c r="F3" s="1"/>
+      <x:c r="G3" s="6" t="str">
+        <x:v>RELIANCE.NS</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="6" t="str">
@@ -364,6 +371,9 @@
       </x:c>
       <x:c r="E4" s="1"/>
       <x:c r="F4" s="1"/>
+      <x:c r="G4" s="6" t="str">
+        <x:v>RELIANCE.NS</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="1"/>
@@ -410,6 +420,9 @@
       <x:c r="F8" s="4" t="str">
         <x:v>Sell Date</x:v>
       </x:c>
+      <x:c r="G8" s="4" t="str">
+        <x:v>Yahoo Finance Code</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="6" t="str">
@@ -425,6 +438,9 @@
       </x:c>
       <x:c r="F9" s="7" t="d">
         <x:v>2026-03-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="str">
+        <x:v>RELIANCE.NS</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -461,7 +477,7 @@
     </x:row>
     <x:row r="5" ht="44" customHeight="1">
       <x:c r="A5" s="10" t="str">
-        <x:v>Stock: enter the stock symbol or name, such as RELIANCE. Use the import preview to confirm or correct the matched stock code.</x:v>
+        <x:v>Stock: enter the stock symbol or name. Yahoo Finance Code is required on every row, e.g. RELIANCE.NS (NSE) or 500325.BO (BSE).</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="44" customHeight="1">

</xml_diff>